<commit_message>
code adjusement, remove badge role pilotage, comprendre, analyser. integration de couleur de theme
</commit_message>
<xml_diff>
--- a/liste_flat_indicateurs.xlsx
+++ b/liste_flat_indicateurs.xlsx
@@ -536,7 +536,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:I39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -546,7 +546,8 @@
     <col width="40" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="6"/>
     <col width="40" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -577,17 +578,22 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>description_indicateur</t>
+          <t>description_indicateur_utilisateur</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>objectif</t>
+          <t>objectif_INFO</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>priorite</t>
+          <t>objectif_AMC</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Analyse_multicriteres</t>
         </is>
       </c>
     </row>
@@ -617,15 +623,20 @@
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>Quantité d’eau que la source peut fournir (référence de période sèche).</t>
+          <t>Estimation de la quantité d'eau prélevable au niveau de la ressource en respectant un objectif de gestion visant à laisser en tout temps 50% de la ressource s'écouler vers l'aval, notamment en période d'étiage médian. Cette information s'appuie sur la ressource "Hydrométrie – Stations DAVAR / Bassins versants aux limnimètres" produite par la DAVAR, qui regroupe les métadonnées des stations de jaugeage et les limnimètres territoriaux.</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>Comparer la capacité des captages à fournir de l’eau en période contrainte (sécheresse, inondation, glissement de terrain) afin d’identifier les ressources les plus robustes ou les plus limitées.</t>
+          <t>Informer sur la quantité d’eau mobilisable par le captage en conditions normales et contraintes afin d’évaluer la disponibilité potentielle de la ressource en eau.</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>Évaluer l’impact sur la disponibilité de la ressource en eau, une faible capacité de production augmentant la criticité en situation de tension.</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
@@ -657,15 +668,20 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>Nombre de personnes alimentées par la ressource.</t>
+          <t>Estimation du nombre d'habitants rattachés à l'unité de distribution (UD) alimentés par la ressource. Le calcul s'appuie sur les fichiers administratifs internes de suivi des abonnés issus de la base de données de l'unité de distribution de la DASS.</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>Comparer les captages selon le nombre de personnes dépendantes afin d’identifier les ressources les plus stratégiques pour l’alimentation en eau.</t>
+          <t>Informer sur le nombre d’habitants dépendants du captage afin de caractériser l’importance des usages associés.</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>Évaluer l’importance stratégique du captage pour l’alimentation en eau, une population élevée augmentant la criticité.</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
@@ -697,15 +713,20 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Statut d’utilisation (actif, secours, abandonné).</t>
+          <t>Établit s'il s'agit d'une ressource principale (actif), d'une ressource utilisée occasionnellement (secours) ou d'une ressource abandonnée. Cette donnée mobilise la ressource "Captages d'eau" produite par la DAVAR décrivant l'état d'utilisation opérationnelle de chaque point d'eau.</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>Distinguer les captages selon leur statut afin de contextualiser leur valeur dans la comparaison.</t>
+          <t>Informer sur le rôle opérationnel du captage (actif, secours, abandonné) afin de contextualiser son utilisation.</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>Évaluer l’importance fonctionnelle du captage dans le système d’alimentation en eau, un captage principal augmentant la criticité.</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
@@ -713,7 +734,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
@@ -725,27 +746,32 @@
           <t>Enjeux AEP</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>Niveau infrastructures</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>Longueur réseau</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>Longueur totale des canalisations d’eau potable.</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
-        <is>
-          <t>Comparer l’importance des infrastructures dépendantes de chaque captage afin d’identifier ceux dont la défaillance aurait le plus d’impact.</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Importance captage</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Établissements public sensibles</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Estimation du nombre d'établissements sensibles (hôpitaux, dispensaires, écoles) rattachés à l'unité de distribution alimentés par la ressource. Aucun fournisseur de ces données n’est pour le moment défini et ces données pourraient être issues des inventaires des services publics et des infrastructures prioritaires dépendantes de la ressource en eau. Ces données sont rattaché au Unité de Distribution (voir CDE ou DASS).</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Informer sur la présence d’établissements sensibles dépendants du captage afin de caractériser les usages prioritaires.</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Évaluer l’importance stratégique de la ressource en eau pour les services essentiels, un nombre élevé augmentant la criticité.</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
@@ -753,7 +779,7 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
@@ -772,20 +798,25 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Capacité réservoir</t>
+          <t>Longueur réseau</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Quantité d’eau pouvant être stockée pour faire face aux besoins.</t>
+          <t>Établit la longueur approximative des réseaux d'adduction et de distribution de l'unité de distribution (UD) associée à la ressource. Ces données proviennent des registres de l'unité de distribution gérés par la DASS, initialement destinés à une vocation administrative interne décrivant les infrastructures linéaires.</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Comparer la capacité de stockage associée aux captages afin d’identifier les systèmes les plus résilients face aux aléas.</t>
+          <t>Informer sur l’étendue des réseaux d’adduction et de distribution dépendants du captage afin de caractériser l’importance des infrastructures alimentées.</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>Évaluer l’importance stratégique des infrastructures dépendantes de la ressource en eau, un réseau étendu augmentant la criticité en cas de défaillance.</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
@@ -793,7 +824,7 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
@@ -805,27 +836,32 @@
           <t>Enjeux AEP</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>Sécurité sanitaire et règlementaire</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>Traitement</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>Type de traitement appliqué à l’eau avant distribution.</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>Comparer le niveau de sécurisation sanitaire des captages afin d’identifier ceux présentant des risques pour l’alimentation en eau potable.</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Niveau infrastructures</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>Capacité réservoir</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Établit le volume de stockage des réservoirs d'eau de l'unité de distribution (UD) associée à la ressource. Cet indicateur mobilise les informations administratives internes de la DASS relatives aux capacités de stockage d'eau potable des unités de distribution.</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>Informer sur la capacité de stockage d’eau associée au captage afin de comprendre la capacité de régulation du système.</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>Évaluer la résilience de la ressource en eau face aux aléas, un faible stockage augmentant la criticité.</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
@@ -833,7 +869,7 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
@@ -852,20 +888,25 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>Statut AODPE</t>
+          <t>Traitement</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>Présence ou non d’une autorisation officielle.</t>
+          <t>Définit le type de traitement d'eau associé à la ressource en eau avant sa mise en distribution. La donnée est issue des fichiers de l'unité de distribution de la DASS, qui décrivent le fonctionnement technique et sanitaire des installations de traitement.</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>Comparer les captages selon leur niveau de conformité réglementaire afin d’identifier les situations à risque.</t>
+          <t>Informer sur le niveau de traitement appliqué à l’eau avant distribution afin de caractériser la sécurisation sanitaire du captage.</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>Évaluer les risques liés à la qualité de la ressource en eau, une absence ou insuffisance de traitement augmentant la criticité sanitaire.</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
@@ -873,7 +914,7 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
@@ -892,20 +933,25 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>Statut PPE</t>
+          <t>Statut AODPE</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>Statut de protection légal et spatial autour de la ressource d’eau potable.</t>
+          <t>Établit le statut de l'autorisation de prélèvement d'eau de la ressource et les informations associées, comme le numéro d'arrêté et le volume autorisé. Cet indicateur de conformité s'appuie sur la base "AODPE" de la DAVAR, qui centralise les données administratives relatives aux autorisations.</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>Comparer les captages selon leur niveau de protection afin d’identifier ceux les plus exposés aux pressions.</t>
+          <t>Informer sur le statut réglementaire du prélèvement d’eau afin de caractériser la conformité administrative du captage.</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>Évaluer les risques réglementaires liés à la ressource en eau, une absence d’autorisation augmentant la criticité.</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
@@ -913,7 +959,7 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
@@ -932,20 +978,25 @@
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>Statut du foncier</t>
+          <t>Statut PPE</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>Typologie permet d'identifier le type de propriétaire de la parcelle</t>
+          <t>Établit le statut du périmètre de protection établi pour la ressource en fonction du type d'arrêté le définissant (État, GNC ou Aucun). L'indicateur exploite la ressource "Périmètres de protection des eaux" de la DAVAR pour refléter l'état d'avancement des dossiers administratifs de protection réglementaire.</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>Comparer les captages selon leur implantation sur dans le cadastre afin de déterminer de potentiel vulnérabilité réglementaire</t>
+          <t>Informer sur le niveau de protection réglementaire du captage afin de comprendre son niveau de sécurisation face aux pressions.</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>Évaluer la vulnérabilité de la ressource en eau face aux pressions extérieures, une absence de protection augmentant la criticité.</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
@@ -953,7 +1004,7 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
@@ -965,27 +1016,32 @@
           <t>Enjeux AEP</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
-        <is>
-          <t>Vulnérabilité structurelle</t>
-        </is>
-      </c>
-      <c r="E11" s="7" t="inlineStr">
-        <is>
-          <t>Interconnexion</t>
-        </is>
-      </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>Présence de connexions avec d’autres réseaux d’eau.</t>
-        </is>
-      </c>
-      <c r="G11" s="7" t="inlineStr">
-        <is>
-          <t>Comparer le niveau de dépendance des captages à une ressource unique afin d’identifier ceux pouvant bénéficier d’un captage de secours.</t>
-        </is>
-      </c>
-      <c r="H11" s="7" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>Sécurité sanitaire et règlementaire</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>Statut du foncier</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>Établit la nature foncière de la parcelle occupée par le prélèvement d'eau, distinguant les terrains publics, privés ou coutumiers. Cet indicateur utilise la ressource "Parcelle cadastrale" produite par la DITTT pour identifier le propriétaire du terrain d'implantation.</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>Informer sur le contexte foncier du captage afin de caractériser les conditions d’accès et de gestion.</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>Évaluer les contraintes foncières pouvant affecter la gestion de la ressource en eau, certaines situations augmentant la criticité.</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
@@ -993,7 +1049,7 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
@@ -1012,20 +1068,25 @@
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>Type ouvrage</t>
+          <t>Interconnexion</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>Type de captage (captage, forage, tranchée drainante).</t>
+          <t>Établit la présence de connexions avec d'autres unités de distribution (UD) pouvant servir de secours. Cet indicateur utilise les informations de l'unité de distribution gérées par la DASS pour identifier la présence de liaisons physiques entre les réseaux d'eau.</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>Comparer les captages selon leur vulnérabilité intrinsèque liée à leur nature {un captage superficiel est considéré comme plus vulnérable qu'un forage profond dans les calculs de criticité)</t>
+          <t>Informer sur la présence ou l’absence de connexions avec d’autres réseaux d’eau afin de comprendre les possibilités de secours.</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Évaluer la sécurisation de la ressource en eau, l’absence d’interconnexion augmentant la criticité en cas de défaillance.</t>
+        </is>
+      </c>
+      <c r="I12" s="7" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
@@ -1033,39 +1094,44 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>105</v>
+        <v>9</v>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
           <t>Enjeu</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
-        <is>
-          <t>Enjeux Environnementaux</t>
-        </is>
-      </c>
-      <c r="D13" s="9" t="inlineStr">
-        <is>
-          <t>Zone naturelle</t>
-        </is>
-      </c>
-      <c r="E13" s="9" t="inlineStr">
-        <is>
-          <t>Occupation sol (couvert végétal)</t>
-        </is>
-      </c>
-      <c r="F13" s="9" t="inlineStr">
-        <is>
-          <t>Superficie des intersections avec des zones de couvert végétal</t>
-        </is>
-      </c>
-      <c r="G13" s="9" t="inlineStr">
-        <is>
-          <t>Caractériser la présence de couvert végétal comme indicateur de bon état écologique du milieu.</t>
-        </is>
-      </c>
-      <c r="H13" s="9" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Enjeux AEP</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Vulnérabilité structurelle</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>Type ouvrage</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr">
+        <is>
+          <t>Établit le type de ressource en eaux en fonction de l'ouvrage, tel que le captage superficiel, le forage ou la tranchée drainante. L'indicateur s'appuie sur la base "Captages d'eau" de la DAVAR répertoriant les caractéristiques techniques des ouvrages de prélèvement.</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>Informer sur le type d’ouvrage de captage afin de caractériser ses caractéristiques techniques.</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>Évaluer la vulnérabilité intrinsèque de la ressource en eau, certains types d’ouvrages augmentant la criticité.</t>
+        </is>
+      </c>
+      <c r="I13" s="7" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
@@ -1073,7 +1139,7 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
@@ -1092,20 +1158,25 @@
       </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
-          <t>Occupation sol (couvert forestier)</t>
+          <t>Occupation sol (couvert végétal)</t>
         </is>
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
-          <t>Superficie des intersections avec des zones de couverture forestière non perturbée et dégradée</t>
+          <t>Mesure la superficie des intersections avec des zones de couvert végétal. L'indicateur croise le MOS 2014 (OEIL/GOUV) et la ressource Dynamic World (Google) pour fournir une description détaillée des classes de végétation et de leur évolution.</t>
         </is>
       </c>
       <c r="G14" s="9" t="inlineStr">
         <is>
-          <t>Évaluer l'état de la couverture forestière, protectrice de la ressource en eau.</t>
+          <t>Informer sur la couverture végétale du bassin versant afin de caractériser l’état du milieu.</t>
         </is>
       </c>
       <c r="H14" s="9" t="inlineStr">
+        <is>
+          <t>Évaluer la capacité du milieu à limiter les transferts vers la ressource en eau, une faible couverture augmentant la criticité.</t>
+        </is>
+      </c>
+      <c r="I14" s="9" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
@@ -1113,7 +1184,7 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
@@ -1125,35 +1196,40 @@
           <t>Enjeux Environnementaux</t>
         </is>
       </c>
-      <c r="D15" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Zones protégés </t>
-        </is>
-      </c>
-      <c r="E15" s="10" t="inlineStr">
-        <is>
-          <t>Zones UNESCO</t>
-        </is>
-      </c>
-      <c r="F15" s="10" t="inlineStr">
-        <is>
-          <t>Superficie des intersections avec les zones inscrites au patrimoine mondial de l'UNESCO</t>
-        </is>
-      </c>
-      <c r="G15" s="10" t="inlineStr">
-        <is>
-          <t>Comparer les bassins versants AEP entre eux par rapport à leur taux de couverture par une zone UNESCO</t>
-        </is>
-      </c>
-      <c r="H15" s="10" t="inlineStr">
-        <is>
-          <t>non</t>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>Zone naturelle</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>Occupation sol (couvert forestier)</t>
+        </is>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>Mesure la superficie des intersections avec des zones de couverture forestière non perturbée et dégradée. La donnée est basée sur la "Cartographie des surfaces forestières" (TMF) décrivant l'étendue de la forêt tropicale humide sans distinction des classes dynamiques.</t>
+        </is>
+      </c>
+      <c r="G15" s="9" t="inlineStr">
+        <is>
+          <t>Informer sur la couverture forestière afin de caractériser le niveau de protection naturelle.</t>
+        </is>
+      </c>
+      <c r="H15" s="9" t="inlineStr">
+        <is>
+          <t>Évaluer le rôle protecteur de la forêt sur la ressource en eau, une faible couverture augmentant la criticité.</t>
+        </is>
+      </c>
+      <c r="I15" s="9" t="inlineStr">
+        <is>
+          <t>oui</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
@@ -1172,28 +1248,33 @@
       </c>
       <c r="E16" s="10" t="inlineStr">
         <is>
-          <t>Zones protégées provinciales</t>
+          <t>Zones UNESCO</t>
         </is>
       </c>
       <c r="F16" s="10" t="inlineStr">
         <is>
-          <t>Superficie des intersections avec parcs, réserves</t>
+          <t>Mesure la superficie des intersections avec les zones inscrites au patrimoine mondial de l'UNESCO. L'indicateur exploite la couche du CEN décrivant les zones terrestres tampons qui alimentent les zones marines classées au patrimoine mondial.</t>
         </is>
       </c>
       <c r="G16" s="10" t="inlineStr">
         <is>
-          <t>Comparer les bassins versants AEP entre eux par rapport à leur taux de couverture par une zone protégée provinciale</t>
+          <t>Informer sur la présence de zones inscrites au patrimoine mondial de l’UNESCO dans le bassin versant afin de caractériser les enjeux environnementaux, patrimoniaux et les opportunités de valorisation et de financement associées.</t>
         </is>
       </c>
       <c r="H16" s="10" t="inlineStr">
         <is>
-          <t>non</t>
+          <t>Évaluer l’effet de la présence de zones UNESCO sur la ressource en eau en termes de préservation du milieu et de potentiel d’accès à des financements internationaux, une forte couverture pouvant réduire la criticité environnementale tout en augmentant l’intérêt stratégique du captage.</t>
+        </is>
+      </c>
+      <c r="I16" s="10" t="inlineStr">
+        <is>
+          <t>oui</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
@@ -1212,28 +1293,33 @@
       </c>
       <c r="E17" s="10" t="inlineStr">
         <is>
-          <t>KBA / ZICO</t>
+          <t>Zones protégées provinciales</t>
         </is>
       </c>
       <c r="F17" s="10" t="inlineStr">
         <is>
-          <t>Superficie des intersections avec les zones d'intérêt biologique et biodiversité spécifique</t>
+          <t>Mesure la superficie des intersections avec les parcs et réserves provinciales en Nouvelle-Calédonie. La donnée compile les fichiers des Aires Protégées produits par les trois provinces (Sud, Nord, Îles) pour identifier les périmètres de conservation du milieu naturel.</t>
         </is>
       </c>
       <c r="G17" s="10" t="inlineStr">
         <is>
-          <t>Comparer les bassins versants AEP entre eux par rapport à leur taux de couverture par une zone KBA/ZICO</t>
+          <t>Informer sur la présence de zones protégées provinciales afin de caractériser le niveau de protection environnementale du bassin versant ainsi que les opportunités de gestion et de financement associées.</t>
         </is>
       </c>
       <c r="H17" s="10" t="inlineStr">
         <is>
-          <t>non</t>
+          <t>Évaluer l’effet des dispositifs de protection réglementaire sur la préservation de la ressource en eau et sur le potentiel de mobilisation de financements, une forte présence contribuant à réduire la criticité liée aux pressions et à renforcer l’intérêt stratégique du territoire.</t>
+        </is>
+      </c>
+      <c r="I17" s="10" t="inlineStr">
+        <is>
+          <t>oui</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
@@ -1252,60 +1338,70 @@
       </c>
       <c r="E18" s="10" t="inlineStr">
         <is>
-          <t>Espèces rares et menacées dont forêt sèche</t>
+          <t>KBA / ZICO</t>
         </is>
       </c>
       <c r="F18" s="10" t="inlineStr">
         <is>
-          <t>Superficie des intersections des patchs de forêt sèche additionné aux zones potentielles de présence d’éspèces rares et menacées</t>
+          <t>Mesure la superficie des intersections avec les zones d'intérêt biologique et de biodiversité spécifique. Cet indicateur est issu de la ressource "Zones clés de biodiversité" du CEN, s'appuyant sur les standards internationaux de l'UICN pour localiser les zones d'intérêt majeur.</t>
         </is>
       </c>
       <c r="G18" s="10" t="inlineStr">
         <is>
-          <t>Comparer les bassins versants AEP entre eux par rapport à leur taux de couverture par des patch d’espèces rares et menacées dont les forêt sèches.</t>
+          <t>Informer sur la présence de zones à forte valeur écologique reconnues internationalement (KBA/ZICO) afin de caractériser les enjeux de biodiversité et les opportunités de financement associées.</t>
         </is>
       </c>
       <c r="H18" s="10" t="inlineStr">
         <is>
-          <t>non</t>
+          <t>Évaluer le rôle de ces zones dans la préservation de la ressource en eau et dans l’accès à des dispositifs de financement environnementaux, une forte présence pouvant réduire la criticité écologique tout en augmentant l’intérêt stratégique du bassin versant.</t>
+        </is>
+      </c>
+      <c r="I18" s="10" t="inlineStr">
+        <is>
+          <t>oui</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>107</v>
-      </c>
-      <c r="B19" s="11" t="inlineStr">
-        <is>
-          <t>Menace</t>
-        </is>
-      </c>
-      <c r="C19" s="12" t="inlineStr">
-        <is>
-          <t>MENACES ANTHROPIQUES</t>
-        </is>
-      </c>
-      <c r="D19" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Activités à risque </t>
-        </is>
-      </c>
-      <c r="E19" s="13" t="inlineStr">
-        <is>
-          <t>Occupation sol (surfaces agricoles)</t>
-        </is>
-      </c>
-      <c r="F19" s="13" t="inlineStr">
-        <is>
-          <t>Superficie des intersections avec des zones agricoles par type (terres arables, agropastorales, pépinières, sylviculture)</t>
-        </is>
-      </c>
-      <c r="G19" s="13" t="inlineStr">
-        <is>
-          <t>Mesurer l'emprise agricole, source potentielle de pression sur la qualité et la quantité de la ressource.</t>
-        </is>
-      </c>
-      <c r="H19" s="13" t="inlineStr">
+        <v>104</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Enjeu</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Enjeux Environnementaux</t>
+        </is>
+      </c>
+      <c r="D19" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Zones protégés </t>
+        </is>
+      </c>
+      <c r="E19" s="10" t="inlineStr">
+        <is>
+          <t>Espèces rares et menacées dont forêt sèche</t>
+        </is>
+      </c>
+      <c r="F19" s="10" t="inlineStr">
+        <is>
+          <t>Mesure la superficie des intersections des patchs de forêt sèche additionnée aux zones potentielles de présence d’espèces rares et menacées. L'indicateur fusionne les données "Espèces rares" d'Endemia et les "Indices de vulnérabilité de la forêt sèche" du CEN pour cartographier les écosystèmes fragiles.</t>
+        </is>
+      </c>
+      <c r="G19" s="10" t="inlineStr">
+        <is>
+          <t>Informer sur la présence d’écosystèmes sensibles afin de caractériser les enjeux écologiques du territoire.</t>
+        </is>
+      </c>
+      <c r="H19" s="10" t="inlineStr">
+        <is>
+          <t>Évaluer le rôle des milieux sensibles dans la protection de la ressource en eau, une forte présence réduisant la criticité.</t>
+        </is>
+      </c>
+      <c r="I19" s="10" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
@@ -1313,7 +1409,7 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>300</v>
+        <v>107</v>
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
@@ -1332,20 +1428,25 @@
       </c>
       <c r="E20" s="13" t="inlineStr">
         <is>
-          <t>ICPE</t>
+          <t>Occupation sol (surfaces agricoles)</t>
         </is>
       </c>
       <c r="F20" s="13" t="inlineStr">
         <is>
-          <t>Nombre de sites industriels à risque.</t>
+          <t>Mesure la superficie des intersections avec des zones agricoles par type, incluant les terres arables, agropastorales ou la sylviculture. L'indicateur utilise le Mode d'Occupation du Sol (MOS 2014) de l'OEIL et du Gouvernement pour décrire les classes d'emprise humaine.</t>
         </is>
       </c>
       <c r="G20" s="13" t="inlineStr">
         <is>
-          <t>Comparer les bassins versants selon la densité d’activités à risque afin d’identifier les sources potentielles de pollution.</t>
+          <t>Informer sur l’emprise agricole du territoire afin de caractériser les usages du sol.</t>
         </is>
       </c>
       <c r="H20" s="13" t="inlineStr">
+        <is>
+          <t>Évaluer les pressions diffuses exercées sur la ressource en eau, une forte emprise agricole augmentant la criticité.</t>
+        </is>
+      </c>
+      <c r="I20" s="13" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
@@ -1353,7 +1454,7 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
@@ -1372,20 +1473,25 @@
       </c>
       <c r="E21" s="13" t="inlineStr">
         <is>
-          <t>Zone d’exploitation minière</t>
+          <t>ICPE</t>
         </is>
       </c>
       <c r="F21" s="13" t="inlineStr">
         <is>
-          <t>Surface occupée par les activités minières.</t>
+          <t>Dénombre les sites d'Installations Classées pour la Protection de l'Environnement, incluant les sites industriels, agricoles ou les stations de traitement. L'indicateur compile les bases ICPE de la DIMENC et des provinces Sud, Nord et Îles Loyauté.</t>
         </is>
       </c>
       <c r="G21" s="13" t="inlineStr">
         <is>
-          <t>Comparer les bassins versants selon l’emprise minière afin d’identifier les pressions fortes sur la ressource.</t>
+          <t>Informer sur la présence d’activités à risque afin de caractériser les sources potentielles de pollution.</t>
         </is>
       </c>
       <c r="H21" s="13" t="inlineStr">
+        <is>
+          <t>Évaluer les pressions industrielles sur la ressource en eau, une forte densité augmentant la criticité.</t>
+        </is>
+      </c>
+      <c r="I21" s="13" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
@@ -1393,7 +1499,7 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
@@ -1405,27 +1511,32 @@
           <t>MENACES ANTHROPIQUES</t>
         </is>
       </c>
-      <c r="D22" s="14" t="inlineStr">
-        <is>
-          <t>Infrastructures et usages</t>
-        </is>
-      </c>
-      <c r="E22" s="14" t="inlineStr">
-        <is>
-          <t>Urbanisation</t>
-        </is>
-      </c>
-      <c r="F22" s="14" t="inlineStr">
-        <is>
-          <t>Nombre de bâtiments présents.</t>
-        </is>
-      </c>
-      <c r="G22" s="14" t="inlineStr">
-        <is>
-          <t>Comparer les bassins versants selon leur niveau d’artificialisation afin d’identifier les pressions liées aux activités humaines.</t>
-        </is>
-      </c>
-      <c r="H22" s="14" t="inlineStr">
+      <c r="D22" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Activités à risque </t>
+        </is>
+      </c>
+      <c r="E22" s="13" t="inlineStr">
+        <is>
+          <t>Zone d’exploitation minière</t>
+        </is>
+      </c>
+      <c r="F22" s="13" t="inlineStr">
+        <is>
+          <t>Mesure la surface occupée par les activités minières, définie par les autorisations d'exploiter ou estimée via le MOS 2014. La donnée est issue de la ressource "Exploitation minière" de la DIMENC localisant les centres miniers et usines métallurgiques actifs.</t>
+        </is>
+      </c>
+      <c r="G22" s="13" t="inlineStr">
+        <is>
+          <t>Informer sur l’emprise minière afin de caractériser les activités extractives.</t>
+        </is>
+      </c>
+      <c r="H22" s="13" t="inlineStr">
+        <is>
+          <t>Évaluer les pressions fortes sur la ressource en eau, une emprise élevée augmentant la criticité.</t>
+        </is>
+      </c>
+      <c r="I22" s="13" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
@@ -1433,7 +1544,7 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
@@ -1445,27 +1556,32 @@
           <t>MENACES ANTHROPIQUES</t>
         </is>
       </c>
-      <c r="D23" s="14" t="inlineStr">
-        <is>
-          <t>Infrastructures et usages</t>
-        </is>
-      </c>
-      <c r="E23" s="14" t="inlineStr">
-        <is>
-          <t>Habitations</t>
-        </is>
-      </c>
-      <c r="F23" s="14" t="inlineStr">
-        <is>
-          <t>Nombre de logements.</t>
-        </is>
-      </c>
-      <c r="G23" s="14" t="inlineStr">
-        <is>
-          <t>Comparer les bassins versants selon la densité d’habitat afin d’affiner l’analyse des pressions humaines.</t>
-        </is>
-      </c>
-      <c r="H23" s="14" t="inlineStr">
+      <c r="D23" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Activités à risque </t>
+        </is>
+      </c>
+      <c r="E23" s="13" t="inlineStr">
+        <is>
+          <t>Autres IOTA</t>
+        </is>
+      </c>
+      <c r="F23" s="13" t="inlineStr">
+        <is>
+          <t>Dénombre les installations, ouvrages ou activités (cultures hors sols, dépotoirs) potentiellement impactants mais non soumis à autorisation classique. Cet indicateur utilise les inventaires techniques de terrain pour identifier les pratiques non référencées par ailleurs.</t>
+        </is>
+      </c>
+      <c r="G23" s="13" t="inlineStr">
+        <is>
+          <t>Informer sur la présence d’activités non réglementées afin de caractériser les pressions diffuses.</t>
+        </is>
+      </c>
+      <c r="H23" s="13" t="inlineStr">
+        <is>
+          <t>Évaluer les pressions non contrôlées sur la ressource en eau.</t>
+        </is>
+      </c>
+      <c r="I23" s="13" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
@@ -1473,7 +1589,7 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
@@ -1492,20 +1608,25 @@
       </c>
       <c r="E24" s="14" t="inlineStr">
         <is>
-          <t>Franchissements</t>
+          <t>Urbanisation</t>
         </is>
       </c>
       <c r="F24" s="14" t="inlineStr">
         <is>
-          <t>Nombre d'ouvrages croisant le réseau hydrographique</t>
+          <t>Dénombre les bâtiments présents sur l'aire d'alimentation de la ressource en eau. Utilisant la ressource "Localités et zones bâties" de la DITTT, cet indicateur s'appuie sur la couche géographique des villes, lieux-dits et tribus au 1/50 000e.</t>
         </is>
       </c>
       <c r="G24" s="14" t="inlineStr">
         <is>
-          <t>Identifier les points de franchissement (ponts, buses, gués) comme facteurs de perturbation du réseau hydrographique. Chaque pont, buse ou gué est un point où une pollution routière (hydrocarbures, transport de matières dangereuses) peut entrer directement dans le cours d'eau en amont d'un captage</t>
+          <t>Informer sur la présence de zones urbanisées afin de caractériser l’occupation du sol.</t>
         </is>
       </c>
       <c r="H24" s="14" t="inlineStr">
+        <is>
+          <t>Évaluer l’artificialisation et ses impacts sur la ressource en eau.</t>
+        </is>
+      </c>
+      <c r="I24" s="14" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
@@ -1513,7 +1634,7 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="B25" s="11" t="inlineStr">
         <is>
@@ -1532,20 +1653,25 @@
       </c>
       <c r="E25" s="14" t="inlineStr">
         <is>
-          <t>Linéaire routes</t>
+          <t>Habitations</t>
         </is>
       </c>
       <c r="F25" s="14" t="inlineStr">
         <is>
-          <t>Distance de linéaire total de voiries par type (RT, RP, Piste)</t>
+          <t>Dénombre le nombre de logements (résidences principales et secondaires) sur l'aire d'alimentation. L'indicateur exploite la "Typologie de l'habitat" de l'ISEE, issue du croisement entre le recensement et les zones bâties de la BDTOPO.</t>
         </is>
       </c>
       <c r="G25" s="14" t="inlineStr">
         <is>
-          <t>Mesurer la densité du réseau routier comme indicateur de pression sur les milieux naturels et la ressource en eau. Une forte densité de routes et de pistes (souvent non classées et plus érosives) augmente l'apport de sédiments dans les cours d'eau (turbidité, engrangement) et donne l'accès à des zones sensibles et peut potentiellement provoquer des pollutions.</t>
+          <t>Informer sur la densité d’habitat afin de caractériser les pressions humaines.</t>
         </is>
       </c>
       <c r="H25" s="14" t="inlineStr">
+        <is>
+          <t>Évaluer la pression liée à la densité humaine sur la ressource en eau.</t>
+        </is>
+      </c>
+      <c r="I25" s="14" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
@@ -1553,7 +1679,7 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="B26" s="11" t="inlineStr">
         <is>
@@ -1572,28 +1698,33 @@
       </c>
       <c r="E26" s="14" t="inlineStr">
         <is>
-          <t>Plan d’Urbanisme Directeur</t>
+          <t>Franchissements</t>
         </is>
       </c>
       <c r="F26" s="14" t="inlineStr">
         <is>
-          <t>Type d’occupation et  dynamiques d’aménagement du territoire (zones urbanisées, à urbaniser, naturelles, zones à enjeux, terrain agricole constructible ou non)</t>
+          <t>Dénombre les ouvrages de franchissement (ponts, radiers) situés sur l'aire d'alimentation, chaque pont, buse ou gué est un point où une pollution routière (hydrocarbures, transport de matières dangereuses) peut entrer directement dans le cours d'eau en amont d'un captage. La donnée croise le "Réseau routier" de la DITTT et les inventaires de la DAVAR pour identifier les points de contact avec le réseau hydrographique.</t>
         </is>
       </c>
       <c r="G26" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Comparer les captages selon les perspectives actuelles et futures de l’aménagement du territoire sur la ressource en eau </t>
+          <t>Informer sur la présence d’ouvrages de franchissement afin de caractériser les points de contact avec le réseau hydrographique.</t>
         </is>
       </c>
       <c r="H26" s="14" t="inlineStr">
         <is>
-          <t>non</t>
+          <t>Évaluer les points de vulnérabilité pouvant impacter la ressource en eau.</t>
+        </is>
+      </c>
+      <c r="I26" s="14" t="inlineStr">
+        <is>
+          <t>oui</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>503</v>
+        <v>306</v>
       </c>
       <c r="B27" s="11" t="inlineStr">
         <is>
@@ -1612,20 +1743,25 @@
       </c>
       <c r="E27" s="14" t="inlineStr">
         <is>
-          <t>Nombre de prélèvement AODPE</t>
+          <t>Linéaire routes</t>
         </is>
       </c>
       <c r="F27" s="14" t="inlineStr">
         <is>
-          <t>Nombre de prélèvements d’eau autorisés.</t>
+          <t>Mesure le linéaire total de voiries par type (RT, RP, RC, pistes) intersectant l'aire d'alimentation. Cet indicateur est basé sur la ressource "BDROUTE-NC" de la DITTT décrivant l'ensemble des voies de transport du territoire.</t>
         </is>
       </c>
       <c r="G27" s="14" t="inlineStr">
         <is>
-          <t>Comparer les captages selon le nombre de prélèvements afin d’évaluer la pression d’usage.</t>
+          <t>Informer sur le réseau routier afin de caractériser les infrastructures de transport.</t>
         </is>
       </c>
       <c r="H27" s="14" t="inlineStr">
+        <is>
+          <t>Évaluer les pressions liées aux infrastructures sur la ressource en eau.</t>
+        </is>
+      </c>
+      <c r="I27" s="14" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
@@ -1633,7 +1769,7 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>504</v>
+        <v>307</v>
       </c>
       <c r="B28" s="11" t="inlineStr">
         <is>
@@ -1652,100 +1788,111 @@
       </c>
       <c r="E28" s="14" t="inlineStr">
         <is>
-          <t>Volume des prélèvements AODPE</t>
+          <t>Plan d’Urbanisme Directeur</t>
         </is>
       </c>
       <c r="F28" s="14" t="inlineStr">
         <is>
-          <t>Volume total d’eau prélevé.</t>
+          <t>Mesure la superficie des intersections avec les zones de type d’occupation et les dynamiques d’aménagement futur (zones urbaines, agricoles, naturelles). L'indicateur s'appuie sur les PUD communaux gérés par les provinces définissant les règles d'utilisation du sol.</t>
         </is>
       </c>
       <c r="G28" s="14" t="inlineStr">
         <is>
-          <t>Comparer les captages selon les volumes prélevés afin d’évaluer l’intensité de la pression quantitative.</t>
-        </is>
-      </c>
-      <c r="H28" s="14" t="inlineStr">
-        <is>
-          <t>oui</t>
+          <t>Informer sur les dynamiques d’aménagement du territoire afin de caractériser les évolutions futures.</t>
+        </is>
+      </c>
+      <c r="H28" s="14" t="n">
+        <v/>
+      </c>
+      <c r="I28" s="14" t="inlineStr">
+        <is>
+          <t>non</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>200</v>
+        <v>503</v>
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
           <t>Menace</t>
         </is>
       </c>
-      <c r="C29" s="15" t="inlineStr">
-        <is>
-          <t>MENACES NATURELLES</t>
-        </is>
-      </c>
-      <c r="D29" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Perturbations environnementales </t>
-        </is>
-      </c>
-      <c r="E29" s="16" t="inlineStr">
-        <is>
-          <t>Incendies cumulés</t>
-        </is>
-      </c>
-      <c r="F29" s="16" t="inlineStr">
-        <is>
-          <t>Surface totale touchée par les incendies.</t>
-        </is>
-      </c>
-      <c r="G29" s="16" t="inlineStr">
-        <is>
-          <t>Comparer les bassins versants selon leur historique d’incendies afin d’identifier les milieux les perturbés.</t>
-        </is>
-      </c>
-      <c r="H29" s="16" t="inlineStr">
-        <is>
-          <t>oui</t>
+      <c r="C29" s="12" t="inlineStr">
+        <is>
+          <t>MENACES ANTHROPIQUES</t>
+        </is>
+      </c>
+      <c r="D29" s="14" t="inlineStr">
+        <is>
+          <t>Infrastructures et usages</t>
+        </is>
+      </c>
+      <c r="E29" s="14" t="inlineStr">
+        <is>
+          <t>Nombre de prélèvement AODPE</t>
+        </is>
+      </c>
+      <c r="F29" s="14" t="inlineStr">
+        <is>
+          <t>Dénombre les points de prélèvements d’eau officiellement autorisés situés en amont de la ressource. Cet indicateur utilise la base "AODPE" de la DAVAR centralisant les données administratives des autorisations de prélèvement.</t>
+        </is>
+      </c>
+      <c r="G29" s="14" t="inlineStr">
+        <is>
+          <t>Informer sur le nombre de prélèvements autorisés afin de caractériser les usages.</t>
+        </is>
+      </c>
+      <c r="H29" s="14" t="n">
+        <v/>
+      </c>
+      <c r="I29" s="14" t="inlineStr">
+        <is>
+          <t>non</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>201</v>
+        <v>504</v>
       </c>
       <c r="B30" s="11" t="inlineStr">
         <is>
           <t>Menace</t>
         </is>
       </c>
-      <c r="C30" s="15" t="inlineStr">
-        <is>
-          <t>MENACES NATURELLES</t>
-        </is>
-      </c>
-      <c r="D30" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Perturbations environnementales </t>
-        </is>
-      </c>
-      <c r="E30" s="16" t="inlineStr">
-        <is>
-          <t>Surface érosion</t>
-        </is>
-      </c>
-      <c r="F30" s="16" t="inlineStr">
-        <is>
-          <t>Surface des zones où le sol est abîmé ou fragile.</t>
-        </is>
-      </c>
-      <c r="G30" s="16" t="inlineStr">
-        <is>
-          <t>Comparer les bassins versants selon leur sensibilité à l’érosion afin d’identifier les ressources exposées à des dégradations du milieu.</t>
-        </is>
-      </c>
-      <c r="H30" s="16" t="inlineStr">
+      <c r="C30" s="12" t="inlineStr">
+        <is>
+          <t>MENACES ANTHROPIQUES</t>
+        </is>
+      </c>
+      <c r="D30" s="14" t="inlineStr">
+        <is>
+          <t>Infrastructures et usages</t>
+        </is>
+      </c>
+      <c r="E30" s="14" t="inlineStr">
+        <is>
+          <t>Volume des prélèvements AODPE</t>
+        </is>
+      </c>
+      <c r="F30" s="14" t="inlineStr">
+        <is>
+          <t>Calcule le volume total des autorisations de prélèvement d'eau journalières situées en amont de la ressource. Basé sur la ressource "AODPE" de la DAVAR, cet indicateur cumule les volumes d'eau autorisés par les arrêtés administratifs.</t>
+        </is>
+      </c>
+      <c r="G30" s="14" t="inlineStr">
+        <is>
+          <t>Informer sur les volumes prélevés afin de caractériser l’intensité des usages.</t>
+        </is>
+      </c>
+      <c r="H30" s="14" t="inlineStr">
+        <is>
+          <t>Évaluer la pression quantitative sur la ressource en eau.</t>
+        </is>
+      </c>
+      <c r="I30" s="14" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
@@ -1753,7 +1900,7 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="B31" s="11" t="inlineStr">
         <is>
@@ -1772,20 +1919,25 @@
       </c>
       <c r="E31" s="16" t="inlineStr">
         <is>
-          <t>Terrain nu</t>
+          <t>Incendies cumulés</t>
         </is>
       </c>
       <c r="F31" s="16" t="inlineStr">
         <is>
-          <t>Surface de terrain sans végétation.</t>
+          <t>Mesure la surface totale touchée par les incendies ces dernières années. Cet indicateur exploite la ressource "Zones potentiellement brûlées" de l'OEIL, issue des détections quotidiennes des capteurs satellitaires VIIRS depuis 2012.</t>
         </is>
       </c>
       <c r="G31" s="16" t="inlineStr">
         <is>
-          <t>Comparer les bassins versants selon l’étendue des surfaces dégradées afin d’identifier les zones les plus sensibles aux ruissellement et aux transferts de polluants.</t>
+          <t>Informer sur l’historique des incendies afin de caractériser les perturbations du milieu.</t>
         </is>
       </c>
       <c r="H31" s="16" t="inlineStr">
+        <is>
+          <t>Évaluer l’impact des incendies sur la dégradation de la ressource en eau, une forte surface brûlée augmentant la criticité.</t>
+        </is>
+      </c>
+      <c r="I31" s="16" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
@@ -1793,7 +1945,7 @@
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="B32" s="11" t="inlineStr">
         <is>
@@ -1812,20 +1964,23 @@
       </c>
       <c r="E32" s="16" t="inlineStr">
         <is>
-          <t>Espèces exotiques envahissantes (EEE)</t>
+          <t>Surface érosion</t>
         </is>
       </c>
       <c r="F32" s="16" t="inlineStr">
         <is>
-          <t>Présence d´espèces exotiques envahissantes</t>
+          <t>Identifie la surface des zones où le sol est abîmé ou fragile. L'indicateur s'appuie sur la "Cartographie des formes érosives" de l'OEIL décrivant les zones de sols dégradés identifiées par imagerie très haute résolution (Province Sud).</t>
         </is>
       </c>
       <c r="G32" s="16" t="inlineStr">
         <is>
-          <t>Comparer les bassins versants selon la présence d’espèces envahissantes afin d’identifier des pressions écologiques potentielles.</t>
-        </is>
-      </c>
-      <c r="H32" s="16" t="inlineStr">
+          <t>Informer sur les zones érodées afin de caractériser la dégradation des sols.</t>
+        </is>
+      </c>
+      <c r="H32" s="16" t="n">
+        <v/>
+      </c>
+      <c r="I32" s="16" t="inlineStr">
         <is>
           <t>non</t>
         </is>
@@ -1833,7 +1988,7 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B33" s="11" t="inlineStr">
         <is>
@@ -1845,27 +2000,32 @@
           <t>MENACES NATURELLES</t>
         </is>
       </c>
-      <c r="D33" s="17" t="inlineStr">
-        <is>
-          <t>Sensibilité naturelle</t>
-        </is>
-      </c>
-      <c r="E33" s="17" t="inlineStr">
-        <is>
-          <t>Glissement terrain</t>
-        </is>
-      </c>
-      <c r="F33" s="17" t="inlineStr">
-        <is>
-          <t>Zones exposées aux glissements de terrain.</t>
-        </is>
-      </c>
-      <c r="G33" s="17" t="inlineStr">
-        <is>
-          <t>Comparer les bassins versants selon leur instabilité afin d’identifier les zones à risque pour la ressource.</t>
-        </is>
-      </c>
-      <c r="H33" s="17" t="inlineStr">
+      <c r="D33" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Perturbations environnementales </t>
+        </is>
+      </c>
+      <c r="E33" s="16" t="inlineStr">
+        <is>
+          <t>Terrain nu</t>
+        </is>
+      </c>
+      <c r="F33" s="16" t="inlineStr">
+        <is>
+          <t>Mesure la superficie de terrain sans végétation intersectant l'aire d'alimentation, en excluant les zones d'exploitations minières. La donnée utilise le MOS 2014 (OEIL/GOUV) ou le flux Dynamic World pour identifier les surfaces minérales ou dévégétalisées.</t>
+        </is>
+      </c>
+      <c r="G33" s="16" t="inlineStr">
+        <is>
+          <t>Informer sur la présence de surfaces dévégétalisées afin de caractériser la dégradation du milieu.</t>
+        </is>
+      </c>
+      <c r="H33" s="16" t="inlineStr">
+        <is>
+          <t>Évaluer les transferts de polluants et sédiments vers la ressource en eau, une forte présence augmentant la criticité.</t>
+        </is>
+      </c>
+      <c r="I33" s="16" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
@@ -1873,7 +2033,7 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>401</v>
+        <v>204</v>
       </c>
       <c r="B34" s="11" t="inlineStr">
         <is>
@@ -1885,27 +2045,32 @@
           <t>MENACES NATURELLES</t>
         </is>
       </c>
-      <c r="D34" s="17" t="inlineStr">
-        <is>
-          <t>Sensibilité naturelle</t>
-        </is>
-      </c>
-      <c r="E34" s="17" t="inlineStr">
-        <is>
-          <t>Géologie</t>
-        </is>
-      </c>
-      <c r="F34" s="17" t="inlineStr">
-        <is>
-          <t>Type de sol et de roche. Propriété des sols correspondant (infiltrant / intermédiaire / ruisselant)</t>
-        </is>
-      </c>
-      <c r="G34" s="17" t="inlineStr">
-        <is>
-          <t>Comparer les bassins versants selon les propriétés des sols afin de qualifier leur comportement hydrologique.</t>
-        </is>
-      </c>
-      <c r="H34" s="17" t="inlineStr">
+      <c r="D34" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Perturbations environnementales </t>
+        </is>
+      </c>
+      <c r="E34" s="16" t="inlineStr">
+        <is>
+          <t>Espèces exotiques envahissantes (EEE)</t>
+        </is>
+      </c>
+      <c r="F34" s="16" t="inlineStr">
+        <is>
+          <t>Estimation de la présence de cerfs et de cochons basée sur le comptage des mâchoires. Cet indicateur se base sur les données de l'ANCB, utilisant les bilans régionalisés par commune et les résultats des campagnes de régularisation de la faune.</t>
+        </is>
+      </c>
+      <c r="G34" s="16" t="inlineStr">
+        <is>
+          <t>Informer sur la présence d’espèces envahissantes afin de caractériser les perturbations écologiques.</t>
+        </is>
+      </c>
+      <c r="H34" s="16" t="inlineStr">
+        <is>
+          <t>Évaluer la pression écologique exercée sur la ressource en eau.</t>
+        </is>
+      </c>
+      <c r="I34" s="16" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
@@ -1913,7 +2078,7 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>402</v>
+        <v>203</v>
       </c>
       <c r="B35" s="11" t="inlineStr">
         <is>
@@ -1932,20 +2097,25 @@
       </c>
       <c r="E35" s="17" t="inlineStr">
         <is>
-          <t>Vulnérabilité intrinsèque des eaux souterraines</t>
+          <t>Glissement terrain</t>
         </is>
       </c>
       <c r="F35" s="17" t="inlineStr">
         <is>
-          <t>Niveau de sensibilité naturelle du terrain à laisser passer l’eau.</t>
+          <t>Identifie les zones exposées aux glissements de terrain par la répartition des surfaces d'aléa. L'indicateur mobilise la "Compilation des cartographies d'aléa mouvement de terrain" de la DIMENC décrivant les niveaux d'aléa de très faible à élevé.</t>
         </is>
       </c>
       <c r="G35" s="17" t="inlineStr">
         <is>
-          <t>Comparer les bassins versants selon leur vulnérabilité intrinsèque afin d’identifier les zones les plus sensibles aux transferts.</t>
+          <t>Informer sur les zones à risque de glissement afin de caractériser l’instabilité du terrain.</t>
         </is>
       </c>
       <c r="H35" s="17" t="inlineStr">
+        <is>
+          <t>Évaluer les perturbations potentielles de la ressource en eau liées à l’instabilité des sols.</t>
+        </is>
+      </c>
+      <c r="I35" s="17" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
@@ -1953,7 +2123,7 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>500</v>
+        <v>401</v>
       </c>
       <c r="B36" s="11" t="inlineStr">
         <is>
@@ -1972,60 +2142,156 @@
       </c>
       <c r="E36" s="17" t="inlineStr">
         <is>
-          <t>BBR</t>
+          <t>Géologie</t>
         </is>
       </c>
       <c r="F36" s="17" t="inlineStr">
         <is>
-          <t>Bilan Besoin Ressource, Écart entre l’eau disponible et les besoins.</t>
+          <t>Répartition des surfaces géologiques définissant les propriétés des sols (infiltrant, intermédiaire ou ruisselant). L'indicateur est basé sur la "Géologie au 1/200 000e" de la DIMENC et du BRGM décrivant les formations rocheuses et arcs structuraux.</t>
         </is>
       </c>
       <c r="G36" s="17" t="inlineStr">
         <is>
-          <t>Comparer les bassins versants selon l’équilibre ressource/besoins afin d’identifier les situations de tension ou de déficit.</t>
-        </is>
-      </c>
-      <c r="H36" s="17" t="inlineStr">
-        <is>
-          <t>oui</t>
+          <t>Informer sur les propriétés géologiques des sols afin de caractériser leur comportement hydrologique.</t>
+        </is>
+      </c>
+      <c r="H36" s="17" t="n">
+        <v/>
+      </c>
+      <c r="I36" s="17" t="inlineStr">
+        <is>
+          <t>non</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
+        <v>402</v>
+      </c>
+      <c r="B37" s="11" t="inlineStr">
+        <is>
+          <t>Menace</t>
+        </is>
+      </c>
+      <c r="C37" s="15" t="inlineStr">
+        <is>
+          <t>MENACES NATURELLES</t>
+        </is>
+      </c>
+      <c r="D37" s="17" t="inlineStr">
+        <is>
+          <t>Sensibilité naturelle</t>
+        </is>
+      </c>
+      <c r="E37" s="17" t="inlineStr">
+        <is>
+          <t>Vulnérabilité intrinsèque des eaux souterraines</t>
+        </is>
+      </c>
+      <c r="F37" s="17" t="inlineStr">
+        <is>
+          <t>Mesure le niveau de sensibilité naturelle du terrain à laisser passer l'eau via les aquifères. L'indicateur utilise la base "BDLISA-NC" de la DIMENC décrivant les limites et les caractéristiques hydrogéologiques des formations aquifères.</t>
+        </is>
+      </c>
+      <c r="G37" s="17" t="inlineStr">
+        <is>
+          <t>Informer sur la sensibilité naturelle des aquifères.</t>
+        </is>
+      </c>
+      <c r="H37" s="17" t="inlineStr">
+        <is>
+          <t>Évaluer la vulnérabilité de la ressource en eau aux infiltrations et contaminations.</t>
+        </is>
+      </c>
+      <c r="I37" s="17" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>500</v>
+      </c>
+      <c r="B38" s="11" t="inlineStr">
+        <is>
+          <t>Menace</t>
+        </is>
+      </c>
+      <c r="C38" s="15" t="inlineStr">
+        <is>
+          <t>MENACES NATURELLES</t>
+        </is>
+      </c>
+      <c r="D38" s="17" t="inlineStr">
+        <is>
+          <t>Sensibilité naturelle</t>
+        </is>
+      </c>
+      <c r="E38" s="17" t="inlineStr">
+        <is>
+          <t>BBR</t>
+        </is>
+      </c>
+      <c r="F38" s="17" t="inlineStr">
+        <is>
+          <t>Bilan Besoin Ressource calculant l'écart entre l'eau disponible et les besoins en fonction de la population et de la capacité de production. Issu du "Bilan Besoin Ressource" de la DAVAR, il soustrait les prélèvements autorisés aux débits d'étiage médian (DCE2).</t>
+        </is>
+      </c>
+      <c r="G38" s="17" t="inlineStr">
+        <is>
+          <t>Informer sur l’équilibre entre ressource disponible et besoins.</t>
+        </is>
+      </c>
+      <c r="H38" s="17" t="inlineStr">
+        <is>
+          <t>Évaluer les tensions sur la ressource en eau, un déficit augmentant fortement la criticité.</t>
+        </is>
+      </c>
+      <c r="I38" s="17" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
         <v>501</v>
       </c>
-      <c r="B37" s="11" t="inlineStr">
+      <c r="B39" s="11" t="inlineStr">
         <is>
           <t>Menace</t>
         </is>
       </c>
-      <c r="C37" s="15" t="inlineStr">
+      <c r="C39" s="15" t="inlineStr">
         <is>
           <t>MENACES NATURELLES</t>
         </is>
       </c>
-      <c r="D37" s="17" t="inlineStr">
+      <c r="D39" s="17" t="inlineStr">
         <is>
           <t>Sensibilité naturelle</t>
         </is>
       </c>
-      <c r="E37" s="17" t="inlineStr">
+      <c r="E39" s="17" t="inlineStr">
         <is>
           <t>Pluviométrie</t>
         </is>
       </c>
-      <c r="F37" s="17" t="inlineStr">
-        <is>
-          <t>Quantité de pluie reçue.</t>
-        </is>
-      </c>
-      <c r="G37" s="17" t="inlineStr">
-        <is>
-          <t>Comparer les bassins versants selon les apports en eau afin de contextualiser la disponibilité de la ressource.</t>
-        </is>
-      </c>
-      <c r="H37" s="17" t="inlineStr">
+      <c r="F39" s="17" t="inlineStr">
+        <is>
+          <t>Mesure la quantité de pluie moyenne reçue sur l'aire d'alimentation de la ressource. Cet indicateur exploite les données des stations de Météo France NC fournissant les mesures de précipitations moyennes sur le territoire.</t>
+        </is>
+      </c>
+      <c r="G39" s="17" t="inlineStr">
+        <is>
+          <t>Informer sur les apports en eau liés aux précipitations.</t>
+        </is>
+      </c>
+      <c r="H39" s="17" t="n">
+        <v/>
+      </c>
+      <c r="I39" s="17" t="inlineStr">
         <is>
           <t>non</t>
         </is>

</xml_diff>